<commit_message>
Unify confirmed aliases in duty schedule analysis
</commit_message>
<xml_diff>
--- a/reports/duty_schedule_rules_2026.xlsx
+++ b/reports/duty_schedule_rules_2026.xlsx
@@ -240,7 +240,41 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">월 주간 일반약사</t>
+      <t xml:space="preserve">월</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">주간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일반약사</t>
     </r>
     <r>
       <rPr>
@@ -274,7 +308,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">명 추정</t>
+      <t xml:space="preserve">명</t>
     </r>
     <r>
       <rPr>
@@ -291,6 +325,844 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">유종호와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">윤종호는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동일인으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">윤종호로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통일하며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">야간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·on-call</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">별도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">주 비교 범위</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">구조 안정적인 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4~7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">39</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 날짜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. 1~3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월은 운영변화와 날짜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">버전 이상을 별도 검토</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">검증 결과</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">39</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일에서 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MIX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 제외한 직군</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">근무유형별 자리 수 유지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">변경후 세부</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1~7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">70</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일 주담당 당일중복 없음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">전후 차이</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">표기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">157</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">셀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">주담당교체</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">125+MIX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빈칸보완</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연습자추가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">셀수와 교환사건수는 다름</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">필수와 권장의 경계</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">필수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">구조</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명시사유를 근거로 한 제약후보</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정보실</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명중첩회피는 강한권장으로 두되 필수여부확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">불확정</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">업무자격표 전체</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">감사최소수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, OFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정확산식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">휴식시간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">횟수상한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공정성가중치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월간순번이월</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">원본 보존</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원본</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Excel4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">변경하지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">않음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">따라</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분석표의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">유종호</t>
     </r>
     <r>
@@ -308,624 +1180,58 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">윤종호 동일인 가정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">야간</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·on-call </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">별도</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">주 비교 범위</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">구조 안정적인 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4~7</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">39</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개 날짜</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. 1~3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월은 운영변화와 날짜</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">버전 이상을 별도 검토</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">검증 결과</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">39</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일에서 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">MIX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">를 제외한 직군</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">근무유형별 자리 수 유지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">변경후 세부</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1~7</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">70</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일 주담당 당일중복 없음</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">전후 차이</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">표기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">157</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">셀</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주담당교체</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">125+MIX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">빈칸보완</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30+</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">연습자추가</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">셀수와 교환사건수는 다름</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">필수와 권장의 경계</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">필수</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">구조</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">명시사유를 근거로 한 제약후보</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">정보실</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">명중첩회피는 강한권장으로 두되 필수여부확인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">불확정</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">업무자격표 전체</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">감사최소수</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, OFF</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">정확산식</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">휴식시간</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">횟수상한</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공정성가중치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월간순번이월</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">원본 보존</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">원본 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Excel4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개는 변경하지 않음</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이 파일의 윤종호 표기는 명칭통일 가정임을 인원별 비고에 표시</t>
+      <t xml:space="preserve">윤종호를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">윤종호로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통일해</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">집계</t>
     </r>
     <r>
       <rPr>
@@ -5536,24 +5842,118 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">토요 원문은 유종호</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">동일인 가정 확인 필요</t>
+      <t xml:space="preserve">유종호</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">윤종호</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동일인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">윤종호로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
     </r>
   </si>
   <si>
@@ -6825,15 +7225,66 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">윤종호 동일인 가정</t>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">윤종호</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동일인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료</t>
     </r>
     <r>
       <rPr>
@@ -6850,16 +7301,16 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">원문 그대로는 일반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
+      <t xml:space="preserve">일반약사</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">24</t>
     </r>
     <r>
       <rPr>
@@ -6884,6 +7335,57 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">직원</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·MIX6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">총</t>
     </r>
     <r>
@@ -6893,7 +7395,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">36</t>
+      <t xml:space="preserve">35</t>
     </r>
     <r>
       <rPr>
@@ -7315,25 +7817,25 @@
     <t xml:space="preserve">D01</t>
   </si>
   <si>
-    <t xml:space="preserve">이름 불일치</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">세부 양쪽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2607 </t>
+    <t xml:space="preserve">이름 통일(확인 완료)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원문</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 2607 </t>
     </r>
     <r>
       <rPr>
@@ -7384,24 +7886,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">!F7 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">및 당직순서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
+      <t xml:space="preserve">!F7=</t>
     </r>
     <r>
       <rPr>
@@ -7411,32 +7896,279 @@
       </rPr>
       <t xml:space="preserve">윤종호</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">동일인일 가능성이 높으나 확인 전 자동 병합하지 않기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. 35</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">명은 동일인 가정</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동일인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">따라</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">윤종호로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통일하고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">집계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. 7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일반약사</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">24</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전체</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">35</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명</t>
     </r>
     <r>
       <rPr>

</xml_diff>